<commit_message>
Enhance candidate canonicalization pipeline
</commit_message>
<xml_diff>
--- a/data/output/canonical_profiles.xlsx
+++ b/data/output/canonical_profiles.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>276a5d90-7100-42d0-9b02-9c7c5b9673be</t>
+          <t>5a4cfa69-178e-45f8-8b82-0bc8a9b5a819</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -533,7 +533,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>69be6aaa-e8d9-4ea0-9fd5-30060a4c60e8</t>
+          <t>6fd982e3-aa48-4da8-b54f-f991cd6e8287</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -586,7 +586,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -692,7 +692,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>e3109af2-aef2-4005-b7cb-9bdcb4fb0fcb</t>
+          <t>f298034e-c1b1-4f15-8cf7-f06587453a2b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -745,7 +745,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>eb3657fe-818d-4f46-9c3b-34263f602a0e</t>
+          <t>0c02b5c1-1d19-4589-9985-ebdf87b9779a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -798,53 +798,180 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>swathirtcc27@gmail.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Internboot</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Java; Python; Spring Boot; REST APIs; MySQL; PostgreSQL; AWS; Git; GitHub; Network Security; VAPT; Web Application Security; React</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ad188cf9-82c0-44b4-81f7-21cb10063487</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SWATHI S</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>abineeththangavel@gmail.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Python; Java; Power BI; Flask; Pandas; TensorFlow; Scikit-learn</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0.7308</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Wei Zhang</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>wei.zhang@example.com</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="H11" t="n">
         <v>5.9</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Python; Pandas; TensorFlow; PyTorch; Scikit-learn</t>
         </is>
       </c>
-      <c r="K8" t="n">
+      <c r="K11" t="n">
         <v>0.6917</v>
       </c>
     </row>
@@ -859,7 +986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -887,7 +1014,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>276a5d90-7100-42d0-9b02-9c7c5b9673be</t>
+          <t>5a4cfa69-178e-45f8-8b82-0bc8a9b5a819</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -909,7 +1036,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>276a5d90-7100-42d0-9b02-9c7c5b9673be</t>
+          <t>5a4cfa69-178e-45f8-8b82-0bc8a9b5a819</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -931,7 +1058,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>276a5d90-7100-42d0-9b02-9c7c5b9673be</t>
+          <t>5a4cfa69-178e-45f8-8b82-0bc8a9b5a819</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -953,7 +1080,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>69be6aaa-e8d9-4ea0-9fd5-30060a4c60e8</t>
+          <t>6fd982e3-aa48-4da8-b54f-f991cd6e8287</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -975,7 +1102,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>69be6aaa-e8d9-4ea0-9fd5-30060a4c60e8</t>
+          <t>6fd982e3-aa48-4da8-b54f-f991cd6e8287</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -997,7 +1124,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>69be6aaa-e8d9-4ea0-9fd5-30060a4c60e8</t>
+          <t>6fd982e3-aa48-4da8-b54f-f991cd6e8287</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1019,7 +1146,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1041,7 +1168,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1063,7 +1190,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1085,7 +1212,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1107,7 +1234,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1129,7 +1256,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1151,7 +1278,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1173,7 +1300,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1195,7 +1322,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1217,7 +1344,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1239,7 +1366,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1261,7 +1388,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1283,7 +1410,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1305,7 +1432,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1327,7 +1454,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1349,7 +1476,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1371,7 +1498,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>e3109af2-aef2-4005-b7cb-9bdcb4fb0fcb</t>
+          <t>f298034e-c1b1-4f15-8cf7-f06587453a2b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1393,7 +1520,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>e3109af2-aef2-4005-b7cb-9bdcb4fb0fcb</t>
+          <t>f298034e-c1b1-4f15-8cf7-f06587453a2b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1415,7 +1542,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>e3109af2-aef2-4005-b7cb-9bdcb4fb0fcb</t>
+          <t>f298034e-c1b1-4f15-8cf7-f06587453a2b</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1437,7 +1564,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>eb3657fe-818d-4f46-9c3b-34263f602a0e</t>
+          <t>0c02b5c1-1d19-4589-9985-ebdf87b9779a</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1459,7 +1586,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>eb3657fe-818d-4f46-9c3b-34263f602a0e</t>
+          <t>0c02b5c1-1d19-4589-9985-ebdf87b9779a</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1481,7 +1608,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>eb3657fe-818d-4f46-9c3b-34263f602a0e</t>
+          <t>0c02b5c1-1d19-4589-9985-ebdf87b9779a</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1503,108 +1630,570 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Wei Zhang</t>
+          <t>Swathi S</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Wei Zhang</t>
+          <t>Swathi S</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Pandas</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Wei Zhang</t>
+          <t>Swathi S</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>TensorFlow</t>
+          <t>Spring Boot</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Wei Zhang</t>
+          <t>Swathi S</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PyTorch</t>
+          <t>REST APIs</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MySQL</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>VAPT</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Web Application Security</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Swathi S</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>React</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ad188cf9-82c0-44b4-81f7-21cb10063487</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SWATHI S</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Flask</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Pandas</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TensorFlow</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Scikit-learn</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>Wei Zhang</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Wei Zhang</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Pandas</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Wei Zhang</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>TensorFlow</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Wei Zhang</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>PyTorch</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Wei Zhang</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
         <is>
           <t>Scikit-learn</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1664,7 +2253,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1699,7 +2288,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1734,7 +2323,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1777,7 +2366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1810,7 +2399,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1837,7 +2426,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1864,25 +2453,52 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>ABINEETH T</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sri Krishna Arts and Science College Jun 2023 - Apr 2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Appin Technology, Coimbatore</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Wei Zhang</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Carnegie Mellon University</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Master of Science, Machine Learning</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>2020-06</t>
         </is>
@@ -1899,7 +2515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1927,7 +2543,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>276a5d90-7100-42d0-9b02-9c7c5b9673be</t>
+          <t>5a4cfa69-178e-45f8-8b82-0bc8a9b5a819</t>
         </is>
       </c>
       <c r="B2" t="b">
@@ -1947,7 +2563,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>69be6aaa-e8d9-4ea0-9fd5-30060a4c60e8</t>
+          <t>6fd982e3-aa48-4da8-b54f-f991cd6e8287</t>
         </is>
       </c>
       <c r="B3" t="b">
@@ -1967,7 +2583,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4e2ad209-3c46-4aef-8df9-b841657cef22</t>
+          <t>49895727-f6bc-4435-b4c5-6c3664275f21</t>
         </is>
       </c>
       <c r="B4" t="b">
@@ -1987,7 +2603,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12546258-f05e-4f54-b8fe-7ab0ef42ba22</t>
+          <t>ec58b2f0-938a-455e-914f-b7f2060bc0f4</t>
         </is>
       </c>
       <c r="B5" t="b">
@@ -2007,7 +2623,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>e3109af2-aef2-4005-b7cb-9bdcb4fb0fcb</t>
+          <t>f298034e-c1b1-4f15-8cf7-f06587453a2b</t>
         </is>
       </c>
       <c r="B6" t="b">
@@ -2027,7 +2643,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>eb3657fe-818d-4f46-9c3b-34263f602a0e</t>
+          <t>0c02b5c1-1d19-4589-9985-ebdf87b9779a</t>
         </is>
       </c>
       <c r="B7" t="b">
@@ -2047,7 +2663,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>08200b68-0031-496a-b5f4-0de8246b7ddd</t>
+          <t>d4f15326-1940-4cb4-9506-ace41a292d22</t>
         </is>
       </c>
       <c r="B8" t="b">
@@ -2059,6 +2675,66 @@
         </is>
       </c>
       <c r="D8" t="inlineStr">
+        <is>
+          <t>['No work experience found for candidate']</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ad188cf9-82c0-44b4-81f7-21cb10063487</t>
+        </is>
+      </c>
+      <c r="B9" t="b">
+        <v>0</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>['Missing required field: email']</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>['No work experience found for candidate']</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1727d054-500e-4ad2-bf99-125f9b4a6343</t>
+        </is>
+      </c>
+      <c r="B10" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>['No work experience found for candidate']</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>c0c15c97-41ac-4bd3-beb1-a6aacef9fbd6</t>
+        </is>
+      </c>
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>[]</t>
         </is>

</xml_diff>